<commit_message>
atualizei os dados do FY26 da MSFT
</commit_message>
<xml_diff>
--- a/analise_eua/tecnologia/microsoft/msft_indicators.xlsx
+++ b/analise_eua/tecnologia/microsoft/msft_indicators.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE10"/>
+  <dimension ref="A1:AE11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -589,856 +589,951 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B2" t="n">
-        <v>36.1</v>
+        <v>20.72</v>
       </c>
       <c r="C2" t="n">
-        <v>36.1</v>
+        <v>20.72</v>
       </c>
       <c r="D2" t="n">
-        <v>2.77</v>
+        <v>4.83</v>
       </c>
       <c r="E2" t="n">
-        <v>162681</v>
+        <v>193771</v>
       </c>
       <c r="F2" t="n">
-        <v>36.15</v>
+        <v>40.31</v>
       </c>
       <c r="G2" t="n">
-        <v>10.7</v>
+        <v>6.26</v>
       </c>
       <c r="H2" t="n">
-        <v>3675915820</v>
+        <v>2771165580</v>
       </c>
       <c r="I2" t="n">
-        <v>112184</v>
+        <v>128813</v>
       </c>
       <c r="J2" t="n">
-        <v>94565</v>
+        <v>76843</v>
       </c>
       <c r="K2" t="n">
-        <v>17619</v>
+        <v>51970</v>
       </c>
       <c r="L2" t="n">
-        <v>0.11</v>
+        <v>0.27</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="N2" t="n">
-        <v>22.7</v>
+        <v>14.57</v>
       </c>
       <c r="O2" t="n">
-        <v>29.65</v>
+        <v>30.23</v>
       </c>
       <c r="P2" t="n">
-        <v>23.42</v>
+        <v>21.54</v>
       </c>
       <c r="Q2" t="n">
-        <v>136162</v>
+        <v>182935</v>
       </c>
       <c r="R2" t="n">
-        <v>-72599</v>
+        <v>-139500</v>
       </c>
       <c r="S2" t="n">
-        <v>-51699</v>
+        <v>-52546</v>
       </c>
       <c r="T2" t="n">
-        <v>71611</v>
+        <v>66987</v>
       </c>
       <c r="U2" t="n">
-        <v>64551</v>
+        <v>115948</v>
       </c>
       <c r="V2" t="n">
-        <v>30398</v>
+        <v>77414</v>
       </c>
       <c r="W2" t="n">
-        <v>32488</v>
+        <v>35562</v>
       </c>
       <c r="X2" t="n">
-        <v>62886</v>
+        <v>112976</v>
       </c>
       <c r="Y2" t="n">
-        <v>49913</v>
+        <v>38885</v>
       </c>
       <c r="Z2" t="n">
-        <v>40.1</v>
+        <v>55.36</v>
       </c>
       <c r="AA2" t="n">
-        <v>50066</v>
+        <v>62629</v>
       </c>
       <c r="AB2" t="n">
-        <v>63065</v>
+        <v>57007</v>
       </c>
       <c r="AC2" t="n">
-        <v>3.24</v>
+        <v>3.56</v>
       </c>
       <c r="AD2" t="n">
-        <v>23.65</v>
+        <v>19.77</v>
       </c>
       <c r="AE2" t="n">
-        <v>18420</v>
+        <v>22271</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B3" t="n">
-        <v>37.18</v>
+        <v>36.02</v>
       </c>
       <c r="C3" t="n">
-        <v>37.18</v>
+        <v>36.02</v>
       </c>
       <c r="D3" t="n">
-        <v>2.69</v>
+        <v>2.78</v>
       </c>
       <c r="E3" t="n">
-        <v>131720</v>
+        <v>162681</v>
       </c>
       <c r="F3" t="n">
-        <v>35.96</v>
+        <v>36.15</v>
       </c>
       <c r="G3" t="n">
-        <v>12.21</v>
+        <v>10.68</v>
       </c>
       <c r="H3" t="n">
-        <v>3276996690</v>
+        <v>3667962510</v>
       </c>
       <c r="I3" t="n">
-        <v>91159</v>
+        <v>112184</v>
       </c>
       <c r="J3" t="n">
-        <v>75543</v>
+        <v>94565</v>
       </c>
       <c r="K3" t="n">
-        <v>15616</v>
+        <v>17619</v>
       </c>
       <c r="L3" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="M3" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="N3" t="n">
-        <v>25</v>
+        <v>22.66</v>
       </c>
       <c r="O3" t="n">
-        <v>32.83</v>
+        <v>29.65</v>
       </c>
       <c r="P3" t="n">
-        <v>24.96</v>
+        <v>23.42</v>
       </c>
       <c r="Q3" t="n">
-        <v>118548</v>
+        <v>136162</v>
       </c>
       <c r="R3" t="n">
-        <v>-96970</v>
+        <v>-72599</v>
       </c>
       <c r="S3" t="n">
-        <v>-37757</v>
+        <v>-51699</v>
       </c>
       <c r="T3" t="n">
-        <v>74071</v>
+        <v>71611</v>
       </c>
       <c r="U3" t="n">
-        <v>44477</v>
+        <v>64551</v>
       </c>
       <c r="V3" t="n">
-        <v>22190</v>
+        <v>30398</v>
       </c>
       <c r="W3" t="n">
-        <v>29510</v>
+        <v>32488</v>
       </c>
       <c r="X3" t="n">
-        <v>51700</v>
+        <v>62886</v>
       </c>
       <c r="Y3" t="n">
-        <v>34448</v>
+        <v>49913</v>
       </c>
       <c r="Z3" t="n">
-        <v>27.96</v>
+        <v>40.1</v>
       </c>
       <c r="AA3" t="n">
-        <v>53107</v>
+        <v>50066</v>
       </c>
       <c r="AB3" t="n">
-        <v>64378</v>
+        <v>63065</v>
       </c>
       <c r="AC3" t="n">
-        <v>2.93</v>
+        <v>3.24</v>
       </c>
       <c r="AD3" t="n">
-        <v>24.7</v>
+        <v>23.65</v>
       </c>
       <c r="AE3" t="n">
-        <v>17254</v>
+        <v>18420</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B4" t="n">
-        <v>34.31</v>
+        <v>37.1</v>
       </c>
       <c r="C4" t="n">
-        <v>34.3</v>
+        <v>37.1</v>
       </c>
       <c r="D4" t="n">
-        <v>2.92</v>
+        <v>2.7</v>
       </c>
       <c r="E4" t="n">
-        <v>102384</v>
+        <v>131720</v>
       </c>
       <c r="F4" t="n">
-        <v>34.15</v>
+        <v>35.96</v>
       </c>
       <c r="G4" t="n">
-        <v>12.04</v>
+        <v>12.18</v>
       </c>
       <c r="H4" t="n">
-        <v>2482421940</v>
+        <v>3269862930</v>
       </c>
       <c r="I4" t="n">
-        <v>79441</v>
+        <v>91159</v>
       </c>
       <c r="J4" t="n">
-        <v>111262</v>
+        <v>75543</v>
       </c>
       <c r="K4" t="n">
-        <v>-31821</v>
+        <v>15616</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.31</v>
+        <v>0.12</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.15</v>
+        <v>0.06</v>
       </c>
       <c r="N4" t="n">
-        <v>24.56</v>
+        <v>24.94</v>
       </c>
       <c r="O4" t="n">
-        <v>35.09</v>
+        <v>32.83</v>
       </c>
       <c r="P4" t="n">
-        <v>25.05</v>
+        <v>24.96</v>
       </c>
       <c r="Q4" t="n">
-        <v>87582</v>
+        <v>118548</v>
       </c>
       <c r="R4" t="n">
-        <v>-22680</v>
+        <v>-96970</v>
       </c>
       <c r="S4" t="n">
-        <v>-43935</v>
+        <v>-37757</v>
       </c>
       <c r="T4" t="n">
-        <v>59475</v>
+        <v>74071</v>
       </c>
       <c r="U4" t="n">
-        <v>28107</v>
+        <v>44477</v>
       </c>
       <c r="V4" t="n">
-        <v>14246</v>
+        <v>22190</v>
       </c>
       <c r="W4" t="n">
-        <v>27195</v>
+        <v>29510</v>
       </c>
       <c r="X4" t="n">
-        <v>41441</v>
+        <v>51700</v>
       </c>
       <c r="Y4" t="n">
-        <v>80108</v>
+        <v>34448</v>
       </c>
       <c r="Z4" t="n">
-        <v>31.71</v>
+        <v>27.96</v>
       </c>
       <c r="AA4" t="n">
-        <v>46918</v>
+        <v>53107</v>
       </c>
       <c r="AB4" t="n">
-        <v>49030</v>
+        <v>64378</v>
       </c>
       <c r="AC4" t="n">
-        <v>2.66</v>
+        <v>2.93</v>
       </c>
       <c r="AD4" t="n">
-        <v>27.36</v>
+        <v>24.7</v>
       </c>
       <c r="AE4" t="n">
-        <v>22245</v>
+        <v>17254</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B5" t="n">
-        <v>25.66</v>
+        <v>34.23</v>
       </c>
       <c r="C5" t="n">
-        <v>25.67</v>
+        <v>34.23</v>
       </c>
       <c r="D5" t="n">
-        <v>3.9</v>
+        <v>2.92</v>
       </c>
       <c r="E5" t="n">
-        <v>97843</v>
+        <v>102384</v>
       </c>
       <c r="F5" t="n">
-        <v>36.69</v>
+        <v>34.15</v>
       </c>
       <c r="G5" t="n">
-        <v>11.21</v>
+        <v>12.01</v>
       </c>
       <c r="H5" t="n">
-        <v>1866728880</v>
+        <v>2477060820</v>
       </c>
       <c r="I5" t="n">
-        <v>78400</v>
+        <v>79441</v>
       </c>
       <c r="J5" t="n">
-        <v>104757</v>
+        <v>111262</v>
       </c>
       <c r="K5" t="n">
-        <v>-26357</v>
+        <v>-31821</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.27</v>
+        <v>-0.31</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.16</v>
+        <v>-0.15</v>
       </c>
       <c r="N5" t="n">
-        <v>19.35</v>
+        <v>24.5</v>
       </c>
       <c r="O5" t="n">
-        <v>43.68</v>
+        <v>35.09</v>
       </c>
       <c r="P5" t="n">
-        <v>29.56</v>
+        <v>25.05</v>
       </c>
       <c r="Q5" t="n">
-        <v>89035</v>
+        <v>87582</v>
       </c>
       <c r="R5" t="n">
-        <v>-30311</v>
+        <v>-22680</v>
       </c>
       <c r="S5" t="n">
-        <v>-58876</v>
+        <v>-43935</v>
       </c>
       <c r="T5" t="n">
-        <v>65149</v>
+        <v>59475</v>
       </c>
       <c r="U5" t="n">
-        <v>23886</v>
+        <v>28107</v>
       </c>
       <c r="V5" t="n">
-        <v>9426</v>
+        <v>14246</v>
       </c>
       <c r="W5" t="n">
-        <v>24512</v>
+        <v>27195</v>
       </c>
       <c r="X5" t="n">
-        <v>33938</v>
+        <v>41441</v>
       </c>
       <c r="Y5" t="n">
-        <v>74602</v>
+        <v>80108</v>
       </c>
       <c r="Z5" t="n">
-        <v>20.28</v>
+        <v>31.71</v>
       </c>
       <c r="AA5" t="n">
-        <v>49033</v>
+        <v>46918</v>
       </c>
       <c r="AB5" t="n">
-        <v>57767</v>
+        <v>49030</v>
       </c>
       <c r="AC5" t="n">
-        <v>2.42</v>
+        <v>2.66</v>
       </c>
       <c r="AD5" t="n">
-        <v>24.93</v>
+        <v>27.36</v>
       </c>
       <c r="AE5" t="n">
-        <v>32696</v>
+        <v>22245</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B6" t="n">
-        <v>32.09</v>
+        <v>25.61</v>
       </c>
       <c r="C6" t="n">
-        <v>32.09</v>
+        <v>25.62</v>
       </c>
       <c r="D6" t="n">
-        <v>3.12</v>
+        <v>3.9</v>
       </c>
       <c r="E6" t="n">
-        <v>81602</v>
+        <v>97843</v>
       </c>
       <c r="F6" t="n">
-        <v>36.45</v>
+        <v>36.69</v>
       </c>
       <c r="G6" t="n">
-        <v>13.85</v>
+        <v>11.18</v>
       </c>
       <c r="H6" t="n">
-        <v>1966295380</v>
+        <v>1862681040</v>
       </c>
       <c r="I6" t="n">
-        <v>82278</v>
+        <v>78400</v>
       </c>
       <c r="J6" t="n">
-        <v>130334</v>
+        <v>104757</v>
       </c>
       <c r="K6" t="n">
-        <v>-48056</v>
+        <v>-26357</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.59</v>
+        <v>-0.27</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.34</v>
+        <v>-0.16</v>
       </c>
       <c r="N6" t="n">
-        <v>24.69</v>
+        <v>19.31</v>
       </c>
       <c r="O6" t="n">
-        <v>43.15</v>
+        <v>43.68</v>
       </c>
       <c r="P6" t="n">
-        <v>26.79</v>
+        <v>29.56</v>
       </c>
       <c r="Q6" t="n">
-        <v>76740</v>
+        <v>89035</v>
       </c>
       <c r="R6" t="n">
-        <v>-27577</v>
+        <v>-30311</v>
       </c>
       <c r="S6" t="n">
-        <v>-48486</v>
+        <v>-58876</v>
       </c>
       <c r="T6" t="n">
-        <v>56118</v>
+        <v>65149</v>
       </c>
       <c r="U6" t="n">
-        <v>20622</v>
+        <v>23886</v>
       </c>
       <c r="V6" t="n">
-        <v>8936</v>
+        <v>9426</v>
       </c>
       <c r="W6" t="n">
-        <v>20716</v>
+        <v>24512</v>
       </c>
       <c r="X6" t="n">
-        <v>29652</v>
+        <v>33938</v>
       </c>
       <c r="Y6" t="n">
-        <v>95749</v>
+        <v>74602</v>
       </c>
       <c r="Z6" t="n">
-        <v>16.68</v>
+        <v>20.28</v>
       </c>
       <c r="AA6" t="n">
-        <v>47499</v>
+        <v>49033</v>
       </c>
       <c r="AB6" t="n">
-        <v>50227</v>
+        <v>57767</v>
       </c>
       <c r="AC6" t="n">
-        <v>2.19</v>
+        <v>2.42</v>
       </c>
       <c r="AD6" t="n">
-        <v>26.96</v>
+        <v>24.93</v>
       </c>
       <c r="AE6" t="n">
-        <v>27385</v>
+        <v>32696</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B7" t="n">
-        <v>33.31</v>
+        <v>32.02</v>
       </c>
       <c r="C7" t="n">
-        <v>33.31</v>
+        <v>32.02</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>3.12</v>
       </c>
       <c r="E7" t="n">
-        <v>65755</v>
+        <v>81602</v>
       </c>
       <c r="F7" t="n">
-        <v>30.96</v>
+        <v>36.45</v>
       </c>
       <c r="G7" t="n">
-        <v>12.47</v>
+        <v>13.82</v>
       </c>
       <c r="H7" t="n">
-        <v>1475198500</v>
+        <v>1962069060</v>
       </c>
       <c r="I7" t="n">
-        <v>82110</v>
+        <v>82278</v>
       </c>
       <c r="J7" t="n">
-        <v>136527</v>
+        <v>130334</v>
       </c>
       <c r="K7" t="n">
-        <v>-54417</v>
+        <v>-48056</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.83</v>
+        <v>-0.59</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.46</v>
+        <v>-0.34</v>
       </c>
       <c r="N7" t="n">
-        <v>23.26</v>
+        <v>24.63</v>
       </c>
       <c r="O7" t="n">
-        <v>37.43</v>
+        <v>43.15</v>
       </c>
       <c r="P7" t="n">
-        <v>22.06</v>
+        <v>26.79</v>
       </c>
       <c r="Q7" t="n">
-        <v>60675</v>
+        <v>76740</v>
       </c>
       <c r="R7" t="n">
-        <v>-12223</v>
+        <v>-27577</v>
       </c>
       <c r="S7" t="n">
-        <v>-46031</v>
+        <v>-48486</v>
       </c>
       <c r="T7" t="n">
-        <v>45234</v>
+        <v>56118</v>
       </c>
       <c r="U7" t="n">
-        <v>15441</v>
+        <v>20622</v>
       </c>
       <c r="V7" t="n">
-        <v>2645</v>
+        <v>8936</v>
       </c>
       <c r="W7" t="n">
-        <v>19269</v>
+        <v>20716</v>
       </c>
       <c r="X7" t="n">
-        <v>21914</v>
+        <v>29652</v>
       </c>
       <c r="Y7" t="n">
-        <v>109605</v>
+        <v>95749</v>
       </c>
       <c r="Z7" t="n">
-        <v>9.31</v>
+        <v>16.68</v>
       </c>
       <c r="AA7" t="n">
-        <v>34646</v>
+        <v>47499</v>
       </c>
       <c r="AB7" t="n">
-        <v>40100</v>
+        <v>50227</v>
       </c>
       <c r="AC7" t="n">
-        <v>1.99</v>
+        <v>2.19</v>
       </c>
       <c r="AD7" t="n">
-        <v>34.18</v>
+        <v>26.96</v>
       </c>
       <c r="AE7" t="n">
-        <v>22968</v>
+        <v>27385</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B8" t="n">
-        <v>24.65</v>
+        <v>33.24</v>
       </c>
       <c r="C8" t="n">
-        <v>24.67</v>
+        <v>33.24</v>
       </c>
       <c r="D8" t="n">
-        <v>4.05</v>
+        <v>3.01</v>
       </c>
       <c r="E8" t="n">
-        <v>54641</v>
+        <v>65755</v>
       </c>
       <c r="F8" t="n">
-        <v>31.18</v>
+        <v>30.96</v>
       </c>
       <c r="G8" t="n">
-        <v>9.449999999999999</v>
+        <v>12.44</v>
       </c>
       <c r="H8" t="n">
-        <v>967181650</v>
+        <v>1472002300</v>
       </c>
       <c r="I8" t="n">
-        <v>86455</v>
+        <v>82110</v>
       </c>
       <c r="J8" t="n">
-        <v>133819</v>
+        <v>136527</v>
       </c>
       <c r="K8" t="n">
-        <v>-47364</v>
+        <v>-54417</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.87</v>
+        <v>-0.83</v>
       </c>
       <c r="M8" t="n">
         <v>-0.46</v>
       </c>
       <c r="N8" t="n">
-        <v>18.57</v>
+        <v>23.21</v>
       </c>
       <c r="O8" t="n">
-        <v>38.35</v>
+        <v>37.43</v>
       </c>
       <c r="P8" t="n">
-        <v>20.4</v>
+        <v>22.06</v>
       </c>
       <c r="Q8" t="n">
-        <v>52185</v>
+        <v>60675</v>
       </c>
       <c r="R8" t="n">
-        <v>-15773</v>
+        <v>-12223</v>
       </c>
       <c r="S8" t="n">
-        <v>-36887</v>
+        <v>-46031</v>
       </c>
       <c r="T8" t="n">
-        <v>38260</v>
+        <v>45234</v>
       </c>
       <c r="U8" t="n">
-        <v>13925</v>
+        <v>15441</v>
       </c>
       <c r="V8" t="n">
-        <v>2243</v>
+        <v>2645</v>
       </c>
       <c r="W8" t="n">
-        <v>16876</v>
+        <v>19269</v>
       </c>
       <c r="X8" t="n">
-        <v>19119</v>
+        <v>21914</v>
       </c>
       <c r="Y8" t="n">
-        <v>106132</v>
+        <v>109605</v>
       </c>
       <c r="Z8" t="n">
-        <v>12.57</v>
+        <v>9.31</v>
       </c>
       <c r="AA8" t="n">
-        <v>30400</v>
+        <v>34646</v>
       </c>
       <c r="AB8" t="n">
-        <v>33745</v>
+        <v>40100</v>
       </c>
       <c r="AC8" t="n">
-        <v>1.8</v>
+        <v>1.99</v>
       </c>
       <c r="AD8" t="n">
-        <v>35.2</v>
+        <v>34.18</v>
       </c>
       <c r="AE8" t="n">
-        <v>19543</v>
+        <v>22968</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B9" t="n">
-        <v>42.43</v>
+        <v>24.6</v>
       </c>
       <c r="C9" t="n">
-        <v>42.47</v>
+        <v>24.61</v>
       </c>
       <c r="D9" t="n">
-        <v>2.35</v>
+        <v>4.06</v>
       </c>
       <c r="E9" t="n">
-        <v>45319</v>
+        <v>54641</v>
       </c>
       <c r="F9" t="n">
-        <v>15.02</v>
+        <v>31.18</v>
       </c>
       <c r="G9" t="n">
-        <v>8.5</v>
+        <v>9.43</v>
       </c>
       <c r="H9" t="n">
-        <v>703087000</v>
+        <v>965109940.0000001</v>
       </c>
       <c r="I9" t="n">
-        <v>87508</v>
+        <v>86455</v>
       </c>
       <c r="J9" t="n">
-        <v>133768</v>
+        <v>133819</v>
       </c>
       <c r="K9" t="n">
-        <v>-46260</v>
+        <v>-47364</v>
       </c>
       <c r="L9" t="n">
-        <v>-1.02</v>
+        <v>-0.87</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.5600000000000001</v>
+        <v>-0.46</v>
       </c>
       <c r="N9" t="n">
-        <v>16.53</v>
+        <v>18.53</v>
       </c>
       <c r="O9" t="n">
-        <v>20.03</v>
+        <v>38.35</v>
       </c>
       <c r="P9" t="n">
-        <v>8.9</v>
+        <v>20.4</v>
       </c>
       <c r="Q9" t="n">
-        <v>43884</v>
+        <v>52185</v>
       </c>
       <c r="R9" t="n">
-        <v>-6061</v>
+        <v>-15773</v>
       </c>
       <c r="S9" t="n">
-        <v>-33590</v>
+        <v>-36887</v>
       </c>
       <c r="T9" t="n">
-        <v>32252</v>
+        <v>38260</v>
       </c>
       <c r="U9" t="n">
-        <v>11632</v>
+        <v>13925</v>
       </c>
       <c r="V9" t="n">
-        <v>1371</v>
+        <v>2243</v>
       </c>
       <c r="W9" t="n">
-        <v>14726</v>
+        <v>16876</v>
       </c>
       <c r="X9" t="n">
-        <v>16097</v>
+        <v>19119</v>
       </c>
       <c r="Y9" t="n">
-        <v>111174</v>
+        <v>106132</v>
       </c>
       <c r="Z9" t="n">
-        <v>-92.06999999999999</v>
+        <v>12.57</v>
       </c>
       <c r="AA9" t="n">
-        <v>20323</v>
+        <v>30400</v>
       </c>
       <c r="AB9" t="n">
-        <v>29881</v>
+        <v>33745</v>
       </c>
       <c r="AC9" t="n">
-        <v>1.65</v>
+        <v>1.8</v>
       </c>
       <c r="AD9" t="n">
-        <v>76.63</v>
+        <v>35.2</v>
       </c>
       <c r="AE9" t="n">
-        <v>10721</v>
+        <v>19543</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B10" t="n">
+        <v>42.34</v>
+      </c>
+      <c r="C10" t="n">
+        <v>42.38</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="E10" t="n">
+        <v>45319</v>
+      </c>
+      <c r="F10" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="G10" t="n">
+        <v>8.48</v>
+      </c>
+      <c r="H10" t="n">
+        <v>701547000</v>
+      </c>
+      <c r="I10" t="n">
+        <v>87508</v>
+      </c>
+      <c r="J10" t="n">
+        <v>133768</v>
+      </c>
+      <c r="K10" t="n">
+        <v>-46260</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-1.02</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-0.5600000000000001</v>
+      </c>
+      <c r="N10" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="O10" t="n">
+        <v>20.03</v>
+      </c>
+      <c r="P10" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>43884</v>
+      </c>
+      <c r="R10" t="n">
+        <v>-6061</v>
+      </c>
+      <c r="S10" t="n">
+        <v>-33590</v>
+      </c>
+      <c r="T10" t="n">
+        <v>32252</v>
+      </c>
+      <c r="U10" t="n">
+        <v>11632</v>
+      </c>
+      <c r="V10" t="n">
+        <v>1371</v>
+      </c>
+      <c r="W10" t="n">
+        <v>14726</v>
+      </c>
+      <c r="X10" t="n">
+        <v>16097</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>111174</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>-92.06999999999999</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>20323</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>29881</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>76.63</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>10721</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
         <v>2017</v>
       </c>
-      <c r="B10" t="n">
-        <v>22.87</v>
-      </c>
-      <c r="C10" t="n">
-        <v>22.85</v>
-      </c>
-      <c r="D10" t="n">
-        <v>4.38</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="B11" t="n">
+        <v>22.82</v>
+      </c>
+      <c r="C11" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="E11" t="n">
         <v>31104</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F11" t="n">
         <v>37.08</v>
       </c>
-      <c r="G10" t="n">
-        <v>6.7</v>
-      </c>
-      <c r="H10" t="n">
-        <v>484899600.0000001</v>
-      </c>
-      <c r="I10" t="n">
+      <c r="G11" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="H11" t="n">
+        <v>483892620</v>
+      </c>
+      <c r="I11" t="n">
         <v>86455</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J11" t="n">
         <v>132981</v>
       </c>
-      <c r="K10" t="n">
+      <c r="K11" t="n">
         <v>-46526</v>
       </c>
-      <c r="L10" t="n">
+      <c r="L11" t="n">
         <v>-1.5</v>
       </c>
-      <c r="M10" t="n">
+      <c r="M11" t="n">
         <v>-0.64</v>
       </c>
-      <c r="N10" t="n">
-        <v>17.09</v>
-      </c>
-      <c r="O10" t="n">
+      <c r="N11" t="n">
+        <v>17.05</v>
+      </c>
+      <c r="O11" t="n">
         <v>29.29</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P11" t="n">
         <v>12.83</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q11" t="n">
         <v>39507</v>
       </c>
-      <c r="R10" t="n">
+      <c r="R11" t="n">
         <v>-46781</v>
       </c>
-      <c r="S10" t="n">
+      <c r="S11" t="n">
         <v>8408</v>
       </c>
-      <c r="T10" t="n">
+      <c r="T11" t="n">
         <v>31378</v>
       </c>
-      <c r="U10" t="n">
+      <c r="U11" t="n">
         <v>8129</v>
       </c>
-      <c r="V10" t="n">
+      <c r="V11" t="n">
         <v>-649</v>
       </c>
-      <c r="W10" t="n">
+      <c r="W11" t="n">
         <v>13037</v>
       </c>
-      <c r="X10" t="n">
+      <c r="X11" t="n">
         <v>12388</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="Y11" t="n">
         <v>95324</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="Z11" t="n">
         <v>-22.65</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AA11" t="n">
         <v>57280</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AB11" t="n">
         <v>25067</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AC11" t="n">
         <v>1.53</v>
       </c>
-      <c r="AD10" t="n">
+      <c r="AD11" t="n">
         <v>55.86</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AE11" t="n">
         <v>11788</v>
       </c>
     </row>
@@ -1613,13 +1708,13 @@
         <v>46112</v>
       </c>
       <c r="B2" t="n">
-        <v>86.5</v>
+        <v>86.31999999999999</v>
       </c>
       <c r="C2" t="n">
-        <v>22.22</v>
+        <v>22.17</v>
       </c>
       <c r="D2" t="n">
-        <v>4.5</v>
+        <v>4.51</v>
       </c>
       <c r="E2" t="n">
         <v>39367</v>
@@ -1628,10 +1723,10 @@
         <v>38.34</v>
       </c>
       <c r="G2" t="n">
-        <v>6.63</v>
+        <v>6.62</v>
       </c>
       <c r="H2" t="n">
-        <v>2748882420</v>
+        <v>2742941620</v>
       </c>
       <c r="I2" t="n">
         <v>125432</v>
@@ -1649,7 +1744,7 @@
         <v>0.11</v>
       </c>
       <c r="N2" t="n">
-        <v>17.62</v>
+        <v>17.58</v>
       </c>
       <c r="O2" t="n">
         <v>29.88</v>
@@ -1708,10 +1803,10 @@
         <v>46022</v>
       </c>
       <c r="B3" t="n">
-        <v>93.23</v>
+        <v>93.03</v>
       </c>
       <c r="C3" t="n">
-        <v>30.89</v>
+        <v>30.82</v>
       </c>
       <c r="D3" t="n">
         <v>3.24</v>
@@ -1723,10 +1818,10 @@
         <v>47.32</v>
       </c>
       <c r="G3" t="n">
-        <v>9.17</v>
+        <v>9.15</v>
       </c>
       <c r="H3" t="n">
-        <v>3585606120</v>
+        <v>3577877880</v>
       </c>
       <c r="I3" t="n">
         <v>123278</v>
@@ -1744,7 +1839,7 @@
         <v>0.09</v>
       </c>
       <c r="N3" t="n">
-        <v>24.06</v>
+        <v>24.01</v>
       </c>
       <c r="O3" t="n">
         <v>29.71</v>
@@ -1803,10 +1898,10 @@
         <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>138.18</v>
+        <v>137.88</v>
       </c>
       <c r="C4" t="n">
-        <v>37.49</v>
+        <v>37.4</v>
       </c>
       <c r="D4" t="n">
         <v>2.67</v>
@@ -1818,10 +1913,10 @@
         <v>35.72</v>
       </c>
       <c r="G4" t="n">
-        <v>10.56</v>
+        <v>10.54</v>
       </c>
       <c r="H4" t="n">
-        <v>3834015730</v>
+        <v>3825690770</v>
       </c>
       <c r="I4" t="n">
         <v>120375</v>
@@ -1839,7 +1934,7 @@
         <v>0.05</v>
       </c>
       <c r="N4" t="n">
-        <v>25.02</v>
+        <v>24.97</v>
       </c>
       <c r="O4" t="n">
         <v>28.19</v>
@@ -1898,13 +1993,13 @@
         <v>45747</v>
       </c>
       <c r="B5" t="n">
-        <v>107.24</v>
+        <v>107.01</v>
       </c>
       <c r="C5" t="n">
-        <v>28.7</v>
+        <v>28.64</v>
       </c>
       <c r="D5" t="n">
-        <v>3.48</v>
+        <v>3.49</v>
       </c>
       <c r="E5" t="n">
         <v>33913</v>
@@ -1913,10 +2008,10 @@
         <v>36.86</v>
       </c>
       <c r="G5" t="n">
-        <v>8.6</v>
+        <v>8.58</v>
       </c>
       <c r="H5" t="n">
-        <v>2769462360</v>
+        <v>2763440820</v>
       </c>
       <c r="I5" t="n">
         <v>105019</v>
@@ -1934,7 +2029,7 @@
         <v>0.08</v>
       </c>
       <c r="N5" t="n">
-        <v>21.4</v>
+        <v>21.36</v>
       </c>
       <c r="O5" t="n">
         <v>29.99</v>
@@ -1993,13 +2088,13 @@
         <v>45657</v>
       </c>
       <c r="B6" t="n">
-        <v>128.75</v>
+        <v>128.47</v>
       </c>
       <c r="C6" t="n">
-        <v>33.53</v>
+        <v>33.46</v>
       </c>
       <c r="D6" t="n">
-        <v>2.98</v>
+        <v>2.99</v>
       </c>
       <c r="E6" t="n">
         <v>31097</v>
@@ -2008,10 +2103,10 @@
         <v>34.62</v>
       </c>
       <c r="G6" t="n">
-        <v>10.25</v>
+        <v>10.23</v>
       </c>
       <c r="H6" t="n">
-        <v>3103815100</v>
+        <v>3097123600</v>
       </c>
       <c r="I6" t="n">
         <v>102909</v>
@@ -2029,7 +2124,7 @@
         <v>0.1</v>
       </c>
       <c r="N6" t="n">
-        <v>24.93</v>
+        <v>24.88</v>
       </c>
       <c r="O6" t="n">
         <v>30.59</v>
@@ -2088,13 +2183,13 @@
         <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>128.16</v>
+        <v>127.89</v>
       </c>
       <c r="C7" t="n">
-        <v>34.83</v>
+        <v>34.76</v>
       </c>
       <c r="D7" t="n">
-        <v>2.87</v>
+        <v>2.88</v>
       </c>
       <c r="E7" t="n">
         <v>37935</v>
@@ -2103,10 +2198,10 @@
         <v>37.61</v>
       </c>
       <c r="G7" t="n">
-        <v>10.99</v>
+        <v>10.96</v>
       </c>
       <c r="H7" t="n">
-        <v>3161403560</v>
+        <v>3154639530</v>
       </c>
       <c r="I7" t="n">
         <v>96838</v>
@@ -2124,7 +2219,7 @@
         <v>0.06</v>
       </c>
       <c r="N7" t="n">
-        <v>25.34</v>
+        <v>25.29</v>
       </c>
       <c r="O7" t="n">
         <v>31.55</v>
@@ -2183,13 +2278,13 @@
         <v>45382</v>
       </c>
       <c r="B8" t="n">
-        <v>140.35</v>
+        <v>140.04</v>
       </c>
       <c r="C8" t="n">
-        <v>36.51</v>
+        <v>36.43</v>
       </c>
       <c r="D8" t="n">
-        <v>2.74</v>
+        <v>2.75</v>
       </c>
       <c r="E8" t="n">
         <v>27649</v>
@@ -2198,10 +2293,10 @@
         <v>35.47</v>
       </c>
       <c r="G8" t="n">
-        <v>12.16</v>
+        <v>12.14</v>
       </c>
       <c r="H8" t="n">
-        <v>3079109160</v>
+        <v>3072421260</v>
       </c>
       <c r="I8" t="n">
         <v>85694</v>
@@ -2219,7 +2314,7 @@
         <v>0.02</v>
       </c>
       <c r="N8" t="n">
-        <v>28.1</v>
+        <v>28.04</v>
       </c>
       <c r="O8" t="n">
         <v>33.34</v>
@@ -2278,10 +2373,10 @@
         <v>45291</v>
       </c>
       <c r="B9" t="n">
-        <v>125.62</v>
+        <v>125.35</v>
       </c>
       <c r="C9" t="n">
-        <v>34.87</v>
+        <v>34.8</v>
       </c>
       <c r="D9" t="n">
         <v>2.87</v>
@@ -2293,10 +2388,10 @@
         <v>35.26</v>
       </c>
       <c r="G9" t="n">
-        <v>11.53</v>
+        <v>11.51</v>
       </c>
       <c r="H9" t="n">
-        <v>2747387440</v>
+        <v>2741441840</v>
       </c>
       <c r="I9" t="n">
         <v>84317</v>
@@ -2314,7 +2409,7 @@
         <v>0.01</v>
       </c>
       <c r="N9" t="n">
-        <v>26.6</v>
+        <v>26.55</v>
       </c>
       <c r="O9" t="n">
         <v>33.11</v>
@@ -2373,13 +2468,13 @@
         <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>103.24</v>
+        <v>103.01</v>
       </c>
       <c r="C10" t="n">
-        <v>30.95</v>
+        <v>30.88</v>
       </c>
       <c r="D10" t="n">
-        <v>3.23</v>
+        <v>3.24</v>
       </c>
       <c r="E10" t="n">
         <v>30816</v>
@@ -2388,10 +2483,10 @@
         <v>39.44</v>
       </c>
       <c r="G10" t="n">
-        <v>10.43</v>
+        <v>10.4</v>
       </c>
       <c r="H10" t="n">
-        <v>2301281330</v>
+        <v>2296303900</v>
       </c>
       <c r="I10" t="n">
         <v>79873</v>
@@ -2409,7 +2504,7 @@
         <v>-0.29</v>
       </c>
       <c r="N10" t="n">
-        <v>23.98</v>
+        <v>23.93</v>
       </c>
       <c r="O10" t="n">
         <v>33.79</v>
@@ -2468,13 +2563,13 @@
         <v>45016</v>
       </c>
       <c r="B11" t="n">
-        <v>114.52</v>
+        <v>114.27</v>
       </c>
       <c r="C11" t="n">
-        <v>30.48</v>
+        <v>30.41</v>
       </c>
       <c r="D11" t="n">
-        <v>3.28</v>
+        <v>3.29</v>
       </c>
       <c r="E11" t="n">
         <v>22253</v>
@@ -2483,10 +2578,10 @@
         <v>34.62</v>
       </c>
       <c r="G11" t="n">
-        <v>10.77</v>
+        <v>10.74</v>
       </c>
       <c r="H11" t="n">
-        <v>2095608830</v>
+        <v>2091069820</v>
       </c>
       <c r="I11" t="n">
         <v>79312</v>
@@ -2504,7 +2599,7 @@
         <v>-0.13</v>
       </c>
       <c r="N11" t="n">
-        <v>23.97</v>
+        <v>23.92</v>
       </c>
       <c r="O11" t="n">
         <v>35.45</v>
@@ -2563,13 +2658,13 @@
         <v>44926</v>
       </c>
       <c r="B12" t="n">
-        <v>106.01</v>
+        <v>105.78</v>
       </c>
       <c r="C12" t="n">
-        <v>25.18</v>
+        <v>25.13</v>
       </c>
       <c r="D12" t="n">
-        <v>3.97</v>
+        <v>3.98</v>
       </c>
       <c r="E12" t="n">
         <v>21257</v>
@@ -2578,10 +2673,10 @@
         <v>31.14</v>
       </c>
       <c r="G12" t="n">
-        <v>9.51</v>
+        <v>9.49</v>
       </c>
       <c r="H12" t="n">
-        <v>1741224190</v>
+        <v>1737424180</v>
       </c>
       <c r="I12" t="n">
         <v>77985</v>
@@ -2599,7 +2694,7 @@
         <v>-0.12</v>
       </c>
       <c r="N12" t="n">
-        <v>19.86</v>
+        <v>19.82</v>
       </c>
       <c r="O12" t="n">
         <v>37.94</v>
@@ -2658,13 +2753,13 @@
         <v>44834</v>
       </c>
       <c r="B13" t="n">
-        <v>96.13</v>
+        <v>95.92</v>
       </c>
       <c r="C13" t="n">
-        <v>23.07</v>
+        <v>23.02</v>
       </c>
       <c r="D13" t="n">
-        <v>4.33</v>
+        <v>4.34</v>
       </c>
       <c r="E13" t="n">
         <v>24308</v>
@@ -2673,10 +2768,10 @@
         <v>35.03</v>
       </c>
       <c r="G13" t="n">
-        <v>9.720000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H13" t="n">
-        <v>1687593670</v>
+        <v>1683939740</v>
       </c>
       <c r="I13" t="n">
         <v>77136</v>
@@ -2694,7 +2789,7 @@
         <v>-0.17</v>
       </c>
       <c r="N13" t="n">
-        <v>18.89</v>
+        <v>18.85</v>
       </c>
       <c r="O13" t="n">
         <v>42.38</v>
@@ -2753,13 +2848,13 @@
         <v>44651</v>
       </c>
       <c r="B14" t="n">
-        <v>133.6</v>
+        <v>133.31</v>
       </c>
       <c r="C14" t="n">
-        <v>31.36</v>
+        <v>31.29</v>
       </c>
       <c r="D14" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E14" t="n">
         <v>20641</v>
@@ -2768,10 +2863,10 @@
         <v>33.89</v>
       </c>
       <c r="G14" t="n">
-        <v>13.72</v>
+        <v>13.69</v>
       </c>
       <c r="H14" t="n">
-        <v>2234787250</v>
+        <v>2229991730</v>
       </c>
       <c r="I14" t="n">
         <v>77981</v>
@@ -2789,7 +2884,7 @@
         <v>-0.16</v>
       </c>
       <c r="N14" t="n">
-        <v>26.97</v>
+        <v>26.92</v>
       </c>
       <c r="O14" t="n">
         <v>43.86</v>
@@ -2848,13 +2943,13 @@
         <v>44561</v>
       </c>
       <c r="B15" t="n">
-        <v>129.85</v>
+        <v>129.57</v>
       </c>
       <c r="C15" t="n">
-        <v>34.8</v>
+        <v>34.72</v>
       </c>
       <c r="D15" t="n">
-        <v>2.87</v>
+        <v>2.88</v>
       </c>
       <c r="E15" t="n">
         <v>22531</v>
@@ -2863,10 +2958,10 @@
         <v>36.28</v>
       </c>
       <c r="G15" t="n">
-        <v>15.23</v>
+        <v>15.2</v>
       </c>
       <c r="H15" t="n">
-        <v>2436723400</v>
+        <v>2431394850</v>
       </c>
       <c r="I15" t="n">
         <v>80353</v>
@@ -2884,7 +2979,7 @@
         <v>-0.28</v>
       </c>
       <c r="N15" t="n">
-        <v>30.56</v>
+        <v>30.49</v>
       </c>
       <c r="O15" t="n">
         <v>43.87</v>
@@ -2943,13 +3038,13 @@
         <v>44469</v>
       </c>
       <c r="B16" t="n">
-        <v>99.54000000000001</v>
+        <v>99.31999999999999</v>
       </c>
       <c r="C16" t="n">
-        <v>31.33</v>
+        <v>31.27</v>
       </c>
       <c r="D16" t="n">
-        <v>3.19</v>
+        <v>3.2</v>
       </c>
       <c r="E16" t="n">
         <v>23450</v>
@@ -2958,10 +3053,10 @@
         <v>45.25</v>
       </c>
       <c r="G16" t="n">
-        <v>13.43</v>
+        <v>13.4</v>
       </c>
       <c r="H16" t="n">
-        <v>2040981580</v>
+        <v>2036624040</v>
       </c>
       <c r="I16" t="n">
         <v>78935</v>
@@ -2979,7 +3074,7 @@
         <v>-0.34</v>
       </c>
       <c r="N16" t="n">
-        <v>27.1</v>
+        <v>27.05</v>
       </c>
       <c r="O16" t="n">
         <v>42.98</v>
@@ -3038,13 +3133,13 @@
         <v>44286</v>
       </c>
       <c r="B17" t="n">
-        <v>110.35</v>
+        <v>110.11</v>
       </c>
       <c r="C17" t="n">
-        <v>30.78</v>
+        <v>30.71</v>
       </c>
       <c r="D17" t="n">
-        <v>3.25</v>
+        <v>3.26</v>
       </c>
       <c r="E17" t="n">
         <v>17223</v>
@@ -3053,10 +3148,10 @@
         <v>37.06</v>
       </c>
       <c r="G17" t="n">
-        <v>12.68</v>
+        <v>12.65</v>
       </c>
       <c r="H17" t="n">
-        <v>1705623360</v>
+        <v>1701929250</v>
       </c>
       <c r="I17" t="n">
         <v>81260</v>
@@ -3074,7 +3169,7 @@
         <v>-0.33</v>
       </c>
       <c r="N17" t="n">
-        <v>26.25</v>
+        <v>26.2</v>
       </c>
       <c r="O17" t="n">
         <v>41.31</v>
@@ -3133,10 +3228,10 @@
         <v>44196</v>
       </c>
       <c r="B18" t="n">
-        <v>104.03</v>
+        <v>103.81</v>
       </c>
       <c r="C18" t="n">
-        <v>31.18</v>
+        <v>31.11</v>
       </c>
       <c r="D18" t="n">
         <v>3.21</v>
@@ -3148,10 +3243,10 @@
         <v>35.9</v>
       </c>
       <c r="G18" t="n">
-        <v>12.35</v>
+        <v>12.32</v>
       </c>
       <c r="H18" t="n">
-        <v>1608686150</v>
+        <v>1605210850</v>
       </c>
       <c r="I18" t="n">
         <v>82782</v>
@@ -3169,7 +3264,7 @@
         <v>-0.38</v>
       </c>
       <c r="N18" t="n">
-        <v>26.09</v>
+        <v>26.03</v>
       </c>
       <c r="O18" t="n">
         <v>39.74</v>
@@ -3228,10 +3323,10 @@
         <v>44104</v>
       </c>
       <c r="B19" t="n">
-        <v>109.37</v>
+        <v>109.14</v>
       </c>
       <c r="C19" t="n">
-        <v>32.5</v>
+        <v>32.43</v>
       </c>
       <c r="D19" t="n">
         <v>3.08</v>
@@ -3243,10 +3338,10 @@
         <v>37.39</v>
       </c>
       <c r="G19" t="n">
-        <v>12.31</v>
+        <v>12.29</v>
       </c>
       <c r="H19" t="n">
-        <v>1519479780</v>
+        <v>1516226400</v>
       </c>
       <c r="I19" t="n">
         <v>83216</v>
@@ -3264,7 +3359,7 @@
         <v>-0.44</v>
       </c>
       <c r="N19" t="n">
-        <v>25.73</v>
+        <v>25.67</v>
       </c>
       <c r="O19" t="n">
         <v>38.07</v>

</xml_diff>